<commit_message>
v1.11.0: agrega indicadores de la sección 9 a plan-implementacion.xlsx
Seguimiento de proyectos: nuevas columnas Fecha real de inicio de desarrollo, Fecha real de cierre y Responsable principal (para indicadores de WIP); la matriz de prioridad se corrió de P:S a S:V. Resumen: nueva sección de indicadores (sección 9) — Lead time, Cycle time, Eficiencia de flujo, % de entrega a tiempo, tabla de capacidad por persona con Tope de WIP editable, Índice de concentración y % de cumplimiento de WIP. 49 fórmulas verificadas sin errores.
</commit_message>
<xml_diff>
--- a/docs/plan-implementacion.xlsx
+++ b/docs/plan-implementacion.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="162">
   <si>
     <t xml:space="preserve">Plantilla de implementación por prioridades — cómo usarla</t>
   </si>
@@ -52,25 +52,31 @@
     <t xml:space="preserve">Hoja 'Seguimiento de proyectos'</t>
   </si>
   <si>
-    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Tiene 4 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
+    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado'), en qué momento del ciclo está (columna 'Fase de desarrollo': por iniciar, en desarrollo, en pruebas de calidad, en producción en observación, o en producción estable), y para cuándo se espera (columnas de fecha estimada de inicio y de entrega). Tres columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre' y 'Responsable principal' — alimentan los indicadores automáticos de la hoja 'Resumen'; se llenan a medida que un ítem avanza, no al crear la fila. Tiene 5 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja 'Resumen'</t>
   </si>
   <si>
-    <t xml:space="preserve">Un panel visual que se actualiza solo a partir de las otras dos hojas — no se edita directamente.</t>
+    <t xml:space="preserve">Un panel visual que se actualiza solo a partir de las otras dos hojas — no se edita directamente. Además del avance general, calcula los indicadores de la sección 9 del framework KPS: Lead time, Cycle time, Eficiencia de flujo, % de entrega a tiempo, Índice de concentración y % de cumplimiento de WIP por persona.</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo se calcula la prioridad</t>
   </si>
   <si>
-    <t xml:space="preserve">Se combinan dos preguntas simples: '¿qué tan grave es si esto se atrasa una semana?' (impacto) y '¿qué tan grande es el esfuerzo?' (tamaño). La combinación da la prioridad automáticamente, según la matriz que está al lado de la tabla en la hoja 'Seguimiento de proyectos' (columnas O a R). Impacto alto + esfuerzo pequeño siempre gana — es la forma más simple de evitar que lo urgente-pero-fácil se quede esperando detrás de algo grande y menos importante.</t>
+    <t xml:space="preserve">Se combinan dos preguntas simples: '¿qué tan grave es si esto se atrasa una semana?' (impacto) y '¿qué tan grande es el esfuerzo?' (tamaño). La combinación da la prioridad automáticamente, según la matriz que está al lado de la tabla en la hoja 'Seguimiento de proyectos' (columnas S a V). Impacto alto + esfuerzo pequeño siempre gana — es la forma más simple de evitar que lo urgente-pero-fácil se quede esperando detrás de algo grande y menos importante.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicadores automáticos (sección 9 del framework)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead time y Cycle time se calculan solos a partir de 'Fecha estimada de inicio', 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' de cada proyecto Completado. El Índice de concentración y el % de cumplimiento de WIP salen de contar, por persona, cuántos ítems tiene 'En curso' en la columna 'Responsable principal' — escribe ahí el nombre de cada persona del equipo en la tabla de la hoja 'Resumen' para que el cálculo funcione.</t>
   </si>
   <si>
     <t xml:space="preserve">Qué editar</t>
   </si>
   <si>
-    <t xml:space="preserve">Las celdas en amarillo son las que se completan para cada paso o proyecto nuevo. Las celdas en azul claro son ejemplos — bórralos o reemplázalos cuando empieces a usar la plantilla con datos reales. No toques las columnas de prioridad, ni la hoja 'Resumen': ambas se calculan solas.</t>
+    <t xml:space="preserve">Las celdas en amarillo son las que se completan para cada paso o proyecto nuevo. Las celdas en azul claro son ejemplos — bórralos o reemplázalos cuando empieces a usar la plantilla con datos reales. No toques las columnas de prioridad, la matriz, ni la hoja 'Resumen' — se calculan solas, excepto la celda amarilla de 'Tope de WIP por persona' y la lista de nombres de personas, que sí son editables.</t>
   </si>
   <si>
     <t xml:space="preserve">Sin nombrar herramientas</t>
@@ -217,7 +223,7 @@
     <t xml:space="preserve">Seguimiento de proyectos — de cada solicitud a una prioridad clara</t>
   </si>
   <si>
-    <t xml:space="preserve">Un renglón por proyecto o solicitud. La columna 'Prioridad' se calcula sola — no la edites a mano.</t>
+    <t xml:space="preserve">Un renglón por proyecto o solicitud. La columna 'Prioridad' se calcula sola (matriz a la derecha) — no la edites a mano.</t>
   </si>
   <si>
     <t xml:space="preserve">Proyecto</t>
@@ -244,12 +250,21 @@
     <t xml:space="preserve">Línea de trabajo asignada</t>
   </si>
   <si>
+    <t xml:space="preserve">Fase de desarrollo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fecha estimada de inicio</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha estimada de entrega</t>
   </si>
   <si>
+    <t xml:space="preserve">Fecha real de inicio de desarrollo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable principal (para indicadores de WIP)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Matriz de prioridad (no editar — solo consulta)</t>
   </si>
   <si>
@@ -274,6 +289,9 @@
     <t xml:space="preserve">Producto y experiencia de cliente</t>
   </si>
   <si>
+    <t xml:space="preserve">En desarrollo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Depende de que el área legal apruebe los textos antes de publicar.</t>
   </si>
   <si>
@@ -304,6 +322,9 @@
     <t xml:space="preserve">Datos y reportes internos</t>
   </si>
   <si>
+    <t xml:space="preserve">Por iniciar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Muy alta</t>
   </si>
   <si>
@@ -325,12 +346,36 @@
     <t xml:space="preserve">Plataforma e infraestructura</t>
   </si>
   <si>
-    <t xml:space="preserve">Viene de un diagnóstico ya completado; no es un proyecto nuevo desde cero.</t>
+    <t xml:space="preserve">En pruebas de calidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de un diagnóstico ya completado; en revisión antes de activar los cambios en producción.</t>
   </si>
   <si>
     <t xml:space="preserve">Media</t>
   </si>
   <si>
+    <t xml:space="preserve">Migrar el catálogo de productos a la nueva base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Producto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reduce tiempos de carga que afectan la conversión en el sitio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En producción (ventana de observación)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya salió a producción; se vigila estabilidad antes de cerrar el proyecto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bajo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja</t>
+  </si>
+  <si>
     <t xml:space="preserve">Actualizar librería interna de componentes visuales</t>
   </si>
   <si>
@@ -343,22 +388,16 @@
     <t xml:space="preserve">Es mantenimiento o mejora interna</t>
   </si>
   <si>
-    <t xml:space="preserve">Bajo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bloqueado</t>
   </si>
   <si>
     <t xml:space="preserve">Bloqueado por falta de capacidad disponible esta semana.</t>
   </si>
   <si>
-    <t xml:space="preserve">Baja</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cómo leerla: impacto alto + esfuerzo pequeño siempre gana. Así lo urgente-pero-rápido de resolver no queda esperando detrás de algo grande y menos importante para el negocio.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cómo usar esta hoja: completa un renglón por cada proyecto o solicitud nueva (columnas en amarillo). Las 4 filas en azul claro son ejemplos — bórralas o reemplázalas cuando empieces a registrar proyectos reales. No edites la columna 'Prioridad' ni la matriz de la derecha: se calculan solas.</t>
+    <t xml:space="preserve">Cómo usar esta hoja: completa un renglón por cada proyecto o solicitud nueva (columnas en amarillo). 'Fase de desarrollo' muestra en qué momento del ciclo va cada proyecto (por iniciar, en desarrollo, en pruebas de calidad, en producción en observación, o en producción estable) — junto con 'Estado' y las fechas, responde para cuándo termina y en qué va. 'Fecha real de inicio de desarrollo', 'Fecha real de cierre' y 'Responsable principal' alimentan los indicadores de la hoja 'Resumen' — llénalas a medida que el ítem avanza, no al crearlo. Las 5 filas en azul claro son ejemplos — bórralas o reemplázalas cuando empieces a registrar proyectos reales. No edites la columna 'Prioridad' ni la matriz de la derecha: se calculan solas.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen de avance</t>
@@ -389,18 +428,101 @@
   </si>
   <si>
     <t xml:space="preserve">Completado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En producción (estable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicadores (sección 9 del framework KPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se calculan solos a partir de 'Seguimiento de proyectos' — no edites esta sección, excepto la celda amarilla de Tope de WIP y la lista de personas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope de WIP por persona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editable — el tope individual que acordó el equipo (pilar 2 del framework).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicadores de flujo (sección 9.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead time promedio (días)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha real de cierre − Fecha estimada de inicio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cycle time promedio (días)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha real de cierre − Fecha real de inicio de desarrollo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eficiencia de flujo (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cycle time ÷ Lead time — cuánto del tiempo total fue trabajo activo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de entrega a tiempo (Fecha fija)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De los ítems con 'Tiene fecha límite real' ya Completados, % entregado en la fecha o antes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: los 4 de arriba quedan vacíos hasta que empieces a llenar 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' en 'Seguimiento de proyectos' — al principio solo tienes fechas estimadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacidad y carga por persona — foto de hoy (sección 9.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ítems activos (En curso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Dentro del tope?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">María (ejemplo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juan (ejemplo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total WIP activo del portafolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Índice de concentración (%) — top 2 personas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riesgo de bus factor si supera 40% (sección 9.2 del framework).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de cumplimiento de WIP (personas dentro del tope)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sobre las personas que hoy tienen al menos 1 ítem activo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cómo usar esta tabla: escribe el nombre de cada persona de tu equipo en la columna Persona (las 2 filas en azul son ejemplo, bórralas). El conteo de ítems activos se toma de la columna 'Responsable principal' de 'Seguimiento de proyectos' — usa una sola persona por ítem ahí, no una lista. Esta tabla es una foto de HOY; para medir tendencia real, repite la foto cada semana en el ritual semanal. Si necesitas más de 8 personas, copia el formato de una fila hacia abajo.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
     <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="167" formatCode="0.0&quot; días&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.0\%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -492,6 +614,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF1A1A19"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -536,7 +666,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -551,6 +681,19 @@
       <right style="thin">
         <color rgb="FFD8D7D0"/>
       </right>
+      <top style="thin">
+        <color rgb="FFD8D7D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD8D7D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFD8D7D0"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FFD8D7D0"/>
       </top>
@@ -585,7 +728,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -602,12 +745,16 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -668,6 +815,50 @@
     </xf>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1007,11 +1198,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="21756458"/>
-        <c:axId val="80714581"/>
+        <c:axId val="42176697"/>
+        <c:axId val="98406073"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="21756458"/>
+        <c:axId val="42176697"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1043,7 +1234,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80714581"/>
+        <c:crossAx val="98406073"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1051,7 +1242,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80714581"/>
+        <c:axId val="98406073"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1093,7 +1284,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21756458"/>
+        <c:crossAx val="42176697"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1372,7 +1563,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1386,11 +1577,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="47201558"/>
-        <c:axId val="45384488"/>
+        <c:axId val="86381979"/>
+        <c:axId val="2608457"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="47201558"/>
+        <c:axId val="86381979"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1422,7 +1613,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45384488"/>
+        <c:crossAx val="2608457"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1430,7 +1621,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="45384488"/>
+        <c:axId val="2608457"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1472,7 +1663,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47201558"/>
+        <c:crossAx val="86381979"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1510,10 +1701,10 @@
       <xdr:rowOff>130680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>387720</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>173880</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1656360</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>266040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1542,8 +1733,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>387720</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>173880</xdr:rowOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>266040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1551,7 +1742,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="3101400" y="2666880"/>
+        <a:off x="5497920" y="2666880"/>
         <a:ext cx="5039640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1745,7 +1936,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1772,7 +1963,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1784,7 +1975,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
     </row>
-    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -1796,7 +1987,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -1808,7 +1999,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -1820,7 +2011,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -1832,7 +2023,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
@@ -1844,7 +2035,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
@@ -1856,7 +2047,7 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
@@ -1868,8 +2059,20 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
+    <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B4:F4"/>
@@ -1880,6 +2083,7 @@
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1911,7 +2115,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1924,7 +2128,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1937,257 +2141,257 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>33</v>
       </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="D6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
+      <c r="C8" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
+      <c r="C9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="B10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
+      <c r="C10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
+      <c r="C11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="B12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
+      <c r="C12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="B13" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
+      <c r="C13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="B14" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
+      <c r="C14" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
+      <c r="A16" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2216,7 +2420,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -2229,16 +2433,20 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="16" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2252,10 +2460,14 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2269,342 +2481,438 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8"/>
+        <v>77</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="S4" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F5" s="9" t="s">
+      <c r="A5" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="G5" s="10" t="str">
-        <f aca="false">IFERROR(INDEX($P$6:$R$8,MATCH($E5,$O$6:$O$8,0),MATCH($F5,$P$5:$R$5,0)),"")</f>
+      <c r="B5" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G5" s="11" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E5,$S$6:$S$8,0),MATCH($F5,$T$5:$V$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="O5" s="5" t="s">
+      <c r="H5" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="S5" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="11" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E6,$S$6:$S$8,0),MATCH($F6,$T$5:$V$5,0)),"")</f>
+        <v>Alta</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="S6" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="T6" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="U6" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="V6" s="13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="11" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E7,$S$6:$S$8,0),MATCH($F7,$T$5:$V$5,0)),"")</f>
+        <v>Alta</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="S7" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="T7" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="U7" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="V7" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="P5" s="5" t="s">
+      <c r="E8" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="Q5" s="5" t="s">
+      <c r="F8" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="R5" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+      <c r="G8" s="11" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E8,$S$6:$S$8,0),MATCH($F8,$T$5:$V$5,0)),"")</f>
+        <v>Alta</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G6" s="10" t="str">
-        <f aca="false">IFERROR(INDEX($P$6:$R$8,MATCH($E6,$O$6:$O$8,0),MATCH($F6,$P$5:$R$5,0)),"")</f>
-        <v>Alta</v>
-      </c>
-      <c r="H6" s="9" t="s">
+      <c r="I8" s="10"/>
+      <c r="J8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="S8" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="T8" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="U8" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="V8" s="13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="O6" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="P6" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q6" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="R6" s="12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G7" s="10" t="str">
-        <f aca="false">IFERROR(INDEX($P$6:$R$8,MATCH($E7,$O$6:$O$8,0),MATCH($F7,$P$5:$R$5,0)),"")</f>
-        <v>Alta</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="G9" s="11" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E9,$S$6:$S$8,0),MATCH($F9,$T$5:$V$5,0)),"")</f>
+        <v>Baja</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="P7" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q7" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="R7" s="12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G8" s="10" t="str">
-        <f aca="false">IFERROR(INDEX($P$6:$R$8,MATCH($E8,$O$6:$O$8,0),MATCH($F8,$P$5:$R$5,0)),"")</f>
-        <v>Baja</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="P8" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q8" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="R8" s="12" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($P$6:$R$8,MATCH($E9,$O$6:$O$8,0),MATCH($F9,$P$5:$R$5,0)),"")</f>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="14" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E10,$S$6:$S$8,0),MATCH($F10,$T$5:$V$5,0)),"")</f>
         <v/>
       </c>
-      <c r="H9" s="4"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($P$6:$R$8,MATCH($E10,$O$6:$O$8,0),MATCH($F10,$P$5:$R$5,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H10" s="4"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="O10" s="7" t="s">
-        <v>110</v>
-      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
-      <c r="R10" s="7"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="S10" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+    </row>
+    <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="14" t="str">
+        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E11,$S$6:$S$8,0),MATCH($F11,$T$5:$V$5,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
       <c r="Q11" s="7"/>
-      <c r="R11" s="7"/>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="7"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="O4:R4"/>
-    <mergeCell ref="O10:R13"/>
-    <mergeCell ref="A12:M12"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="S10:V13"/>
+    <mergeCell ref="A13:Q13"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D10" type="list">
+  <dataValidations count="5">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D11" type="list">
       <formula1>"Urgente ahora,Tiene fecha límite real,Puede esperar y priorizarse,Es mantenimiento o mejora interna"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E10" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E11" type="list">
       <formula1>"Alto,Medio,Bajo"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F10" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F11" type="list">
       <formula1>"Pequeño,Mediano,Grande"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J10" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J11" type="list">
       <formula1>"No iniciado,En curso,Completado,Bloqueado"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K11" type="list">
+      <formula1>"Por iniciar,En desarrollo,En pruebas de calidad,En producción (ventana de observación),En producción (estable)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2623,22 +2931,25 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2647,10 +2958,13 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2659,155 +2973,481 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B4" s="8"/>
-      <c r="D4" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" s="8"/>
+      <c r="A4" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="D4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="15" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")/COUNTA('Hoja de ruta'!B5:B14)</f>
         <v>0</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="D5" s="15" t="n">
-        <f aca="false">COUNTA('Seguimiento de proyectos'!A5:A10)</f>
-        <v>4</v>
-      </c>
-      <c r="E5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="D5" s="16" t="n">
+        <f aca="false">COUNTA('Seguimiento de proyectos'!A5:A11)</f>
+        <v>5</v>
+      </c>
+      <c r="E5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>120</v>
+      <c r="A8" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="B9" s="18" t="n">
+      <c r="A9" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="19" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")</f>
         <v>0</v>
       </c>
-      <c r="D9" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$10,"Muy alta")</f>
+      <c r="D9" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Muy alta")</f>
         <v>0</v>
       </c>
-      <c r="G9" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$10,"Completado")</f>
+      <c r="G9" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Completado")</f>
         <v>0</v>
       </c>
+      <c r="J9" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="K9" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"Por iniciar")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="18" t="n">
+      <c r="A10" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="19" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"En curso")</f>
         <v>1</v>
       </c>
-      <c r="D10" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" s="18" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$10,"Alta")</f>
+      <c r="D10" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Alta")</f>
+        <v>4</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"En curso")</f>
         <v>3</v>
       </c>
-      <c r="G10" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" s="20" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$10,"En curso")</f>
-        <v>2</v>
+      <c r="J10" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="K10" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En desarrollo")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="18" t="n">
+      <c r="A11" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="19" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="D11" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="E11" s="18" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$10,"Media")</f>
+      <c r="D11" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Media")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Bloqueado")</f>
+        <v>1</v>
+      </c>
+      <c r="J11" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="20" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$10,"Bloqueado")</f>
+      <c r="K11" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En pruebas de calidad")</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="18" t="n">
+      <c r="A12" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="19" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"No iniciado")</f>
         <v>9</v>
       </c>
-      <c r="D12" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="E12" s="18" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$10,"Baja")</f>
+      <c r="D12" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Baja")</f>
         <v>1</v>
       </c>
-      <c r="G12" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$10,"No iniciado")</f>
+      <c r="G12" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"No iniciado")</f>
         <v>1</v>
       </c>
+      <c r="J12" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="K12" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (ventana de observación)")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J13" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="K13" s="21" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (estable)")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="B22" s="26" t="str">
+        <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$L$5:$L$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="B23" s="26" t="str">
+        <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$O$5:$O$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")),"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="B24" s="27" t="str">
+        <f aca="false">IFERROR(B23/B22*100,"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="B25" s="27" t="str">
+        <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11&lt;='Seguimiento de proyectos'!$M$5:$M$11))/SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;""))*100,"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="24" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="B31" s="19" t="n">
+        <f aca="false">IF($A31="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="19" t="str">
+        <f aca="false">IF($A31="","",IF(B31&lt;=$B$19,"Sí","No"))</f>
+        <v>Sí</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="B32" s="19" t="n">
+        <f aca="false">IF($A32="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="19" t="str">
+        <f aca="false">IF($A32="","",IF(B32&lt;=$B$19,"Sí","No"))</f>
+        <v>Sí</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="31"/>
+      <c r="B33" s="19" t="n">
+        <f aca="false">IF($A33="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A33,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="19" t="str">
+        <f aca="false">IF($A33="","",IF(B33&lt;=$B$19,"Sí","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="31"/>
+      <c r="B34" s="19" t="n">
+        <f aca="false">IF($A34="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A34,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="19" t="str">
+        <f aca="false">IF($A34="","",IF(B34&lt;=$B$19,"Sí","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="31"/>
+      <c r="B35" s="19" t="n">
+        <f aca="false">IF($A35="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A35,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C35" s="19" t="str">
+        <f aca="false">IF($A35="","",IF(B35&lt;=$B$19,"Sí","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="31"/>
+      <c r="B36" s="19" t="n">
+        <f aca="false">IF($A36="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A36,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="19" t="str">
+        <f aca="false">IF($A36="","",IF(B36&lt;=$B$19,"Sí","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="31"/>
+      <c r="B37" s="19" t="n">
+        <f aca="false">IF($A37="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A37,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="19" t="str">
+        <f aca="false">IF($A37="","",IF(B37&lt;=$B$19,"Sí","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="31"/>
+      <c r="B38" s="19" t="n">
+        <f aca="false">IF($A38="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A38,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="19" t="str">
+        <f aca="false">IF($A38="","",IF(B38&lt;=$B$19,"Sí","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B40" s="32" t="n">
+        <f aca="false">SUM($B$31:$B$38)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="B41" s="27" t="str">
+        <f aca="false">IFERROR((LARGE($B$31:$B$38,1)+LARGE($B$31:$B$38,2))/SUM($B$31:$B$38)*100,"")</f>
+        <v/>
+      </c>
+      <c r="C41" s="24" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="B42" s="27" t="str">
+        <f aca="false">IFERROR(SUMPRODUCT(($B$31:$B$38&gt;0)*($B$31:$B$38&lt;=$B$19))/SUMPRODUCT(($B$31:$B$38&gt;0)*1)*100,"")</f>
+        <v/>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8"/>
+      <c r="H44" s="8"/>
+      <c r="I44" s="8"/>
+      <c r="J44" s="8"/>
+      <c r="K44" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+  <mergeCells count="11">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="A5:B6"/>
     <mergeCell ref="D5:E6"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A27:K27"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A44:K44"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
v1.12.0: agrega hoja Roles y gobierno y estado Cancelado
Nueva hoja "Roles y gobierno" (sección 5): 7 roles del framework listados, con una fila de Líder de Flujo de Valor por cada flujo de ejemplo (coherente con "Seguimiento de proyectos"), columnas Titular/Respaldo en amarillo. "Cómo usar" actualizado. "Seguimiento de proyectos": la columna Estado suma el valor "Cancelado", con su conteo en "Resumen". 50 fórmulas verificadas sin errores.
</commit_message>
<xml_diff>
--- a/docs/plan-implementacion.xlsx
+++ b/docs/plan-implementacion.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Hoja de ruta" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Seguimiento de proyectos" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Resumen" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Roles y gobierno" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="187">
   <si>
     <t xml:space="preserve">Plantilla de implementación por prioridades — cómo usarla</t>
   </si>
@@ -52,7 +53,7 @@
     <t xml:space="preserve">Hoja 'Seguimiento de proyectos'</t>
   </si>
   <si>
-    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado'), en qué momento del ciclo está (columna 'Fase de desarrollo': por iniciar, en desarrollo, en pruebas de calidad, en producción en observación, o en producción estable), y para cuándo se espera (columnas de fecha estimada de inicio y de entrega). Tres columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre' y 'Responsable principal' — alimentan los indicadores automáticos de la hoja 'Resumen'; se llenan a medida que un ítem avanza, no al crear la fila. Tiene 5 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
+    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado': incluye 'Cancelado' para lo que se descarta sin completarse), en qué momento del ciclo está (columna 'Fase de desarrollo'), y para cuándo se espera. Tres columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre' y 'Responsable principal' — alimentan los indicadores automáticos de la hoja 'Resumen'. Tiene 5 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja 'Resumen'</t>
@@ -61,6 +62,12 @@
     <t xml:space="preserve">Un panel visual que se actualiza solo a partir de las otras dos hojas — no se edita directamente. Además del avance general, calcula los indicadores de la sección 9 del framework KPS: Lead time, Cycle time, Eficiencia de flujo, % de entrega a tiempo, Índice de concentración y % de cumplimiento de WIP por persona.</t>
   </si>
   <si>
+    <t xml:space="preserve">Hoja 'Roles y gobierno'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El registro de quién tiene cada rol de gobierno del framework (sección 5) y quién es su respaldo nombrado — para que ninguna regla dependa de una sola persona. Trae los 7 roles del framework ya listados, con una fila de 'Líder de Flujo de Valor' por cada flujo de valor (usa los mismos ejemplos de la hoja 'Seguimiento de proyectos'). Completa 'Titular' y 'Respaldo' con los nombres reales de tu equipo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cómo se calcula la prioridad</t>
   </si>
   <si>
@@ -76,7 +83,7 @@
     <t xml:space="preserve">Qué editar</t>
   </si>
   <si>
-    <t xml:space="preserve">Las celdas en amarillo son las que se completan para cada paso o proyecto nuevo. Las celdas en azul claro son ejemplos — bórralos o reemplázalos cuando empieces a usar la plantilla con datos reales. No toques las columnas de prioridad, la matriz, ni la hoja 'Resumen' — se calculan solas, excepto la celda amarilla de 'Tope de WIP por persona' y la lista de nombres de personas, que sí son editables.</t>
+    <t xml:space="preserve">Las celdas en amarillo son las que se completan para cada paso, proyecto o rol nuevo. Las celdas en azul claro son ejemplos — bórralos o reemplázalos cuando empieces a usar la plantilla con datos reales. No toques las columnas de prioridad, la matriz, ni la hoja 'Resumen' — se calculan solas, excepto la celda amarilla de 'Tope de WIP por persona' y la lista de nombres de personas, que sí son editables.</t>
   </si>
   <si>
     <t xml:space="preserve">Sin nombrar herramientas</t>
@@ -430,6 +437,9 @@
     <t xml:space="preserve">Completado</t>
   </si>
   <si>
+    <t xml:space="preserve">Cancelado</t>
+  </si>
+  <si>
     <t xml:space="preserve">En producción (estable)</t>
   </si>
   <si>
@@ -509,6 +519,72 @@
   </si>
   <si>
     <t xml:space="preserve">Cómo usar esta tabla: escribe el nombre de cada persona de tu equipo en la columna Persona (las 2 filas en azul son ejemplo, bórralas). El conteo de ítems activos se toma de la columna 'Responsable principal' de 'Seguimiento de proyectos' — usa una sola persona por ítem ahí, no una lista. Esta tabla es una foto de HOY; para medir tendencia real, repite la foto cada semana en el ritual semanal. Si necesitas más de 8 personas, copia el formato de una fila hacia abajo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roles y gobierno (sección 5 del framework KPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada regla necesita un dueño con nombre, y ese dueño necesita un respaldo nombrado — nunca un punto único de falla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Respaldo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable de Flujo de Portafolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantiene la vista única de capacidad actualizada y decide qué pasa cuando alguien llega a su tope de WIP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprobador de Clase de Servicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Única autoridad para etiquetar un ítem como Expedite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facilitador del Ritual Semanal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corre el triage semanal y verifica la Definición de Listo antes de que algo entre a desarrollo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Representante de Valor de Negocio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todas las líneas (confirmar si se necesita uno por línea)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Única fuente aceptada del componente de valor de negocio (Costo de Demora) del WSJF. Sin su respaldo nombrado, este rol queda con el mismo bus factor que KPS busca eliminar en el resto del equipo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Líder de Flujo de Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guardia Rotativa (Firefighter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Absorbe lo Expedite durante su semana de turno. La rotación es, en sí misma, el mecanismo de respaldo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dueño de Calidad del Flujo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puede bloquear el paso a 'Listo para desplegar' si no cumple la Definición de Hecho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cómo usar esta hoja: completa 'Titular' y 'Respaldo' (columnas en amarillo) para cada rol con el nombre real de la persona de tu equipo. Agrega una fila de 'Líder de Flujo de Valor' por cada flujo de valor adicional que tengas — usa los mismos nombres de flujo que en la columna 'Línea de trabajo asignada' de 'Seguimiento de proyectos', para que ambas hojas hablen el mismo idioma. Ningún rol necesita ser una dedicación de tiempo completo: pueden ser sombreros que ya usan personas del equipo.</t>
   </si>
 </sst>
 </file>
@@ -728,16 +804,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -765,7 +845,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -797,11 +877,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -809,7 +889,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -817,7 +897,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -829,19 +909,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -849,15 +929,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1053,100 +1141,120 @@
             <c:dLbl>
               <c:idx val="0"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="3"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1198,17 +1306,17 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="42176697"/>
-        <c:axId val="98406073"/>
+        <c:axId val="23934050"/>
+        <c:axId val="40487919"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="42176697"/>
+        <c:axId val="23934050"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1234,7 +1342,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98406073"/>
+        <c:crossAx val="40487919"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1242,7 +1350,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98406073"/>
+        <c:axId val="40487919"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1258,7 +1366,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1284,7 +1392,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42176697"/>
+        <c:crossAx val="23934050"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1432,100 +1540,120 @@
             <c:dLbl>
               <c:idx val="0"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:dLbl>
               <c:idx val="3"/>
               <c:txPr>
-                <a:bodyPr wrap="none"/>
+                <a:bodyPr wrap="square"/>
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
                     <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
-              <c:separator> </c:separator>
+              <c:separator>; </c:separator>
             </c:dLbl>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1577,17 +1705,17 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86381979"/>
-        <c:axId val="2608457"/>
+        <c:axId val="10105970"/>
+        <c:axId val="87350264"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86381979"/>
+        <c:axId val="10105970"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1613,7 +1741,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2608457"/>
+        <c:crossAx val="87350264"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1621,7 +1749,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2608457"/>
+        <c:axId val="87350264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1637,7 +1765,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1663,7 +1791,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86381979"/>
+        <c:crossAx val="10105970"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1702,9 +1830,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1656360</xdr:colOff>
+      <xdr:colOff>1655640</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>266040</xdr:rowOff>
+      <xdr:rowOff>265320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1712,8 +1840,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="2666880"/>
-        <a:ext cx="5039640" cy="2519640"/>
+        <a:off x="0" y="2664360"/>
+        <a:ext cx="5038920" cy="2496960"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1732,9 +1860,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>387720</xdr:colOff>
+      <xdr:colOff>387000</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>266040</xdr:rowOff>
+      <xdr:rowOff>265320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1742,8 +1870,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5497920" y="2666880"/>
-        <a:ext cx="5039640" cy="2519640"/>
+        <a:off x="5497920" y="2664360"/>
+        <a:ext cx="5038920" cy="2496960"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1936,143 +2064,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B4:F4"/>
@@ -2084,6 +2224,7 @@
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2103,295 +2244,295 @@
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>30</v>
       </c>
+      <c r="H4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>35</v>
       </c>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
+      <c r="D6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="6" t="s">
+      <c r="B7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="C9" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
+      <c r="C10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
+      <c r="C11" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="C12" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
+      <c r="C13" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="A16" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2423,468 +2564,468 @@
   <dimension ref="A1:V13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="1" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
+      <c r="A1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="I4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="N4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" s="5" t="s">
+      <c r="L4" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="P4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q4" s="5" t="s">
+      <c r="M4" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="N4" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="T4" s="9"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
+      <c r="P4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="S4" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="D5" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="11" t="str">
+      <c r="E5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="G5" s="12" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E5,$S$6:$S$8,0),MATCH($F5,$T$5:$V$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H5" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="K5" s="10" t="s">
+      <c r="H5" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="S5" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="U5" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="V5" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="S5" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="T5" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="U5" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="V5" s="5" t="s">
-        <v>86</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="G6" s="11" t="str">
+      <c r="G6" s="12" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E6,$S$6:$S$8,0),MATCH($F6,$T$5:$V$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H6" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="S6" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="T6" s="13" t="s">
+      <c r="H6" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="U6" s="13" t="s">
+      <c r="I6" s="11"/>
+      <c r="J6" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="V6" s="13" t="s">
-        <v>101</v>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="11"/>
+      <c r="S6" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="T6" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="U6" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="V6" s="14" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="A7" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G7" s="11" t="str">
+      <c r="C7" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G7" s="12" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E7,$S$6:$S$8,0),MATCH($F7,$T$5:$V$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10" t="s">
+      <c r="H7" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="S7" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="T7" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="U7" s="13" t="s">
+      <c r="I7" s="11"/>
+      <c r="J7" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="V7" s="13" t="s">
-        <v>109</v>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
+      <c r="S7" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="T7" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="U7" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="V7" s="14" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="F8" s="10" t="s">
+      <c r="B8" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="11" t="str">
+      <c r="E8" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" s="12" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E8,$S$6:$S$8,0),MATCH($F8,$T$5:$V$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H8" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
-      <c r="S8" s="12" t="s">
+      <c r="H8" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="T8" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="U8" s="13" t="s">
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="V8" s="13" t="s">
-        <v>116</v>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="S8" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="T8" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="U8" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="V8" s="14" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G9" s="11" t="str">
+      <c r="F9" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G9" s="12" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E9,$S$6:$S$8,0),MATCH($F9,$T$5:$V$5,0)),"")</f>
         <v>Baja</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
+      <c r="H9" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="14" t="str">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="15" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E10,$S$6:$S$8,0),MATCH($F10,$T$5:$V$5,0)),"")</f>
         <v/>
       </c>
-      <c r="H10" s="6"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="S10" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="S10" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="T10" s="9"/>
+      <c r="U10" s="9"/>
+      <c r="V10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="14" t="str">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="15" t="str">
         <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E11,$S$6:$S$8,0),MATCH($F11,$T$5:$V$5,0)),"")</f>
         <v/>
       </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
-      <c r="S11" s="8"/>
-      <c r="T11" s="8"/>
-      <c r="U11" s="8"/>
-      <c r="V11" s="8"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="S11" s="9"/>
+      <c r="T11" s="9"/>
+      <c r="U11" s="9"/>
+      <c r="V11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="S12" s="9"/>
+      <c r="T12" s="9"/>
+      <c r="U12" s="9"/>
+      <c r="V12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="8"/>
+      <c r="A13" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="S13" s="9"/>
+      <c r="T13" s="9"/>
+      <c r="U13" s="9"/>
+      <c r="V13" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2908,7 +3049,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J11" type="list">
-      <formula1>"No iniciado,En curso,Completado,Bloqueado"</formula1>
+      <formula1>"No iniciado,En curso,Completado,Bloqueado,Cancelado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K11" type="list">
@@ -2934,506 +3075,513 @@
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="D4" s="9" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="9"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="n">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="D4" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")/COUNTA('Hoja de ruta'!B5:B14)</f>
         <v>0</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="D5" s="16" t="n">
+      <c r="B5" s="16"/>
+      <c r="D5" s="17" t="n">
         <f aca="false">COUNTA('Seguimiento de proyectos'!A5:A11)</f>
         <v>5</v>
       </c>
-      <c r="E5" s="16"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" s="17" t="s">
+      <c r="E5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="D8" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="J8" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="K8" s="17" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="G8" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="H8" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="20" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")</f>
         <v>0</v>
       </c>
-      <c r="D9" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" s="19" t="n">
+      <c r="D9" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="20" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Muy alta")</f>
         <v>0</v>
       </c>
-      <c r="G9" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="H9" s="21" t="n">
+      <c r="G9" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="H9" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Completado")</f>
         <v>0</v>
       </c>
-      <c r="J9" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="K9" s="21" t="n">
+      <c r="J9" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="K9" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"Por iniciar")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="19" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="20" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"En curso")</f>
         <v>1</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="E10" s="19" t="n">
+      <c r="D10" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Alta")</f>
         <v>4</v>
       </c>
-      <c r="G10" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="21" t="n">
+      <c r="G10" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"En curso")</f>
         <v>3</v>
       </c>
-      <c r="J10" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="K10" s="21" t="n">
+      <c r="J10" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="K10" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En desarrollo")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="19" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="20" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="D11" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="E11" s="19" t="n">
+      <c r="D11" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Media")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="H11" s="21" t="n">
+      <c r="G11" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="H11" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Bloqueado")</f>
         <v>1</v>
       </c>
-      <c r="J11" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="K11" s="21" t="n">
+      <c r="J11" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="K11" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En pruebas de calidad")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="19" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="20" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"No iniciado")</f>
         <v>9</v>
       </c>
-      <c r="D12" s="18" t="s">
-        <v>116</v>
-      </c>
-      <c r="E12" s="19" t="n">
+      <c r="D12" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Baja")</f>
         <v>1</v>
       </c>
-      <c r="G12" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="H12" s="21" t="n">
+      <c r="G12" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"No iniciado")</f>
         <v>1</v>
       </c>
-      <c r="J12" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="K12" s="21" t="n">
+      <c r="J12" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="K12" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (ventana de observación)")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J13" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="K13" s="21" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G13" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="H13" s="22" t="n">
+        <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Cancelado")</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="21" t="s">
+        <v>138</v>
+      </c>
+      <c r="K13" s="22" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (estable)")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
-        <v>136</v>
-      </c>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-    </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="B19" s="23" t="n">
+      <c r="A17" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="B19" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="B22" s="26" t="str">
+      <c r="C19" s="25" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B22" s="27" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$L$5:$L$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")),"")</f>
         <v/>
       </c>
-      <c r="C22" s="24" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="B23" s="26" t="str">
+      <c r="C22" s="25" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="B23" s="27" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$O$5:$O$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")),"")</f>
         <v/>
       </c>
-      <c r="C23" s="24" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25" t="s">
-        <v>145</v>
-      </c>
-      <c r="B24" s="27" t="str">
+      <c r="C23" s="25" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B24" s="28" t="str">
         <f aca="false">IFERROR(B23/B22*100,"")</f>
         <v/>
       </c>
-      <c r="C24" s="24" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="B25" s="27" t="str">
+      <c r="C24" s="25" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="B25" s="28" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11&lt;='Seguimiento de proyectos'!$M$5:$M$11))/SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;""))*100,"")</f>
         <v/>
       </c>
-      <c r="C25" s="24" t="s">
-        <v>148</v>
+      <c r="C25" s="25" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
-    </row>
-    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
-        <v>151</v>
-      </c>
-      <c r="B30" s="29" t="s">
+      <c r="A27" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="30" t="s">
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="B31" s="19" t="n">
+      <c r="B30" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="B31" s="20" t="n">
         <f aca="false">IF($A31="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C31" s="19" t="str">
+      <c r="C31" s="20" t="str">
         <f aca="false">IF($A31="","",IF(B31&lt;=$B$19,"Sí","No"))</f>
         <v>Sí</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="B32" s="19" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="20" t="n">
         <f aca="false">IF($A32="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C32" s="19" t="str">
+      <c r="C32" s="20" t="str">
         <f aca="false">IF($A32="","",IF(B32&lt;=$B$19,"Sí","No"))</f>
         <v>Sí</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="31"/>
-      <c r="B33" s="19" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="32"/>
+      <c r="B33" s="20" t="n">
         <f aca="false">IF($A33="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A33,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C33" s="19" t="str">
+      <c r="C33" s="20" t="str">
         <f aca="false">IF($A33="","",IF(B33&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="31"/>
-      <c r="B34" s="19" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="32"/>
+      <c r="B34" s="20" t="n">
         <f aca="false">IF($A34="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A34,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C34" s="19" t="str">
+      <c r="C34" s="20" t="str">
         <f aca="false">IF($A34="","",IF(B34&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="31"/>
-      <c r="B35" s="19" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="32"/>
+      <c r="B35" s="20" t="n">
         <f aca="false">IF($A35="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A35,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C35" s="19" t="str">
+      <c r="C35" s="20" t="str">
         <f aca="false">IF($A35="","",IF(B35&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="31"/>
-      <c r="B36" s="19" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="32"/>
+      <c r="B36" s="20" t="n">
         <f aca="false">IF($A36="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A36,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C36" s="19" t="str">
+      <c r="C36" s="20" t="str">
         <f aca="false">IF($A36="","",IF(B36&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="31"/>
-      <c r="B37" s="19" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="32"/>
+      <c r="B37" s="20" t="n">
         <f aca="false">IF($A37="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A37,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C37" s="19" t="str">
+      <c r="C37" s="20" t="str">
         <f aca="false">IF($A37="","",IF(B37&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="31"/>
-      <c r="B38" s="19" t="n">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="32"/>
+      <c r="B38" s="20" t="n">
         <f aca="false">IF($A38="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A38,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C38" s="19" t="str">
+      <c r="C38" s="20" t="str">
         <f aca="false">IF($A38="","",IF(B38&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17" t="s">
-        <v>156</v>
-      </c>
-      <c r="B40" s="32" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B40" s="33" t="n">
         <f aca="false">SUM($B$31:$B$38)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="25" t="s">
-        <v>157</v>
-      </c>
-      <c r="B41" s="27" t="str">
+    <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="B41" s="28" t="str">
         <f aca="false">IFERROR((LARGE($B$31:$B$38,1)+LARGE($B$31:$B$38,2))/SUM($B$31:$B$38)*100,"")</f>
         <v/>
       </c>
-      <c r="C41" s="24" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="25" t="s">
-        <v>159</v>
-      </c>
-      <c r="B42" s="27" t="str">
+      <c r="C41" s="25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="B42" s="28" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(($B$31:$B$38&gt;0)*($B$31:$B$38&lt;=$B$19))/SUMPRODUCT(($B$31:$B$38&gt;0)*1)*100,"")</f>
         <v/>
       </c>
-      <c r="C42" s="24" t="s">
-        <v>160</v>
+      <c r="C42" s="25" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="8"/>
-      <c r="K44" s="8"/>
+      <c r="A44" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -3458,4 +3606,189 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+    </row>
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="7" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A15:E15"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v1.13.0 — plan-implementacion.xlsx: columna Responsable de QA
Nueva columna "Responsable de QA (para indicadores de WIP)" junto a la de desarrollo en "Seguimiento de proyectos". La tabla de capacidad de "Resumen" (seccion 9.2) ahora suma En curso de ambas columnas. Matriz de prioridad corrida de S-V a T-W; formula de Prioridad actualizada. 50 formulas verificadas sin errores.
</commit_message>
<xml_diff>
--- a/docs/plan-implementacion.xlsx
+++ b/docs/plan-implementacion.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="188">
   <si>
     <t xml:space="preserve">Plantilla de implementación por prioridades — cómo usarla</t>
   </si>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Hoja 'Seguimiento de proyectos'</t>
   </si>
   <si>
-    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado': incluye 'Cancelado' para lo que se descarta sin completarse), en qué momento del ciclo está (columna 'Fase de desarrollo'), y para cuándo se espera. Tres columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre' y 'Responsable principal' — alimentan los indicadores automáticos de la hoja 'Resumen'. Tiene 5 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
+    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado': incluye 'Cancelado' para lo que se descarta sin completarse), en qué momento del ciclo está (columna 'Fase de desarrollo'), y para cuándo se espera. Cuatro columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre', 'Responsable de desarrollo' y 'Responsable de QA' — alimentan los indicadores automáticos de la hoja 'Resumen'. Tiene 5 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja 'Resumen'</t>
@@ -71,13 +71,13 @@
     <t xml:space="preserve">Cómo se calcula la prioridad</t>
   </si>
   <si>
-    <t xml:space="preserve">Se combinan dos preguntas simples: '¿qué tan grave es si esto se atrasa una semana?' (impacto) y '¿qué tan grande es el esfuerzo?' (tamaño). La combinación da la prioridad automáticamente, según la matriz que está al lado de la tabla en la hoja 'Seguimiento de proyectos' (columnas S a V). Impacto alto + esfuerzo pequeño siempre gana — es la forma más simple de evitar que lo urgente-pero-fácil se quede esperando detrás de algo grande y menos importante.</t>
+    <t xml:space="preserve">Se combinan dos preguntas simples: '¿qué tan grave es si esto se atrasa una semana?' (impacto) y '¿qué tan grande es el esfuerzo?' (tamaño). La combinación da la prioridad automáticamente, según la matriz que está al lado de la tabla en la hoja 'Seguimiento de proyectos' (columnas T a W). Impacto alto + esfuerzo pequeño siempre gana — es la forma más simple de evitar que lo urgente-pero-fácil se quede esperando detrás de algo grande y menos importante.</t>
   </si>
   <si>
     <t xml:space="preserve">Indicadores automáticos (sección 9 del framework)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lead time y Cycle time se calculan solos a partir de 'Fecha estimada de inicio', 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' de cada proyecto Completado. El Índice de concentración y el % de cumplimiento de WIP salen de contar, por persona, cuántos ítems tiene 'En curso' en la columna 'Responsable principal' — escribe ahí el nombre de cada persona del equipo en la tabla de la hoja 'Resumen' para que el cálculo funcione.</t>
+    <t xml:space="preserve">Lead time y Cycle time se calculan solos a partir de 'Fecha estimada de inicio', 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' de cada proyecto Completado. El Índice de concentración y el % de cumplimiento de WIP salen de contar, por persona, cuántos ítems tiene 'En curso' sumando la columna 'Responsable de desarrollo' y la columna 'Responsable de QA' — escribe el nombre de cada persona del equipo (desarrollo y QA) en la tabla de la hoja 'Resumen' para que el cálculo funcione.</t>
   </si>
   <si>
     <t xml:space="preserve">Qué editar</t>
@@ -269,7 +269,10 @@
     <t xml:space="preserve">Fecha real de inicio de desarrollo</t>
   </si>
   <si>
-    <t xml:space="preserve">Responsable principal (para indicadores de WIP)</t>
+    <t xml:space="preserve">Responsable de desarrollo (para indicadores de WIP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable de QA (para indicadores de WIP)</t>
   </si>
   <si>
     <t xml:space="preserve">Matriz de prioridad (no editar — solo consulta)</t>
@@ -404,7 +407,7 @@
     <t xml:space="preserve">Cómo leerla: impacto alto + esfuerzo pequeño siempre gana. Así lo urgente-pero-rápido de resolver no queda esperando detrás de algo grande y menos importante para el negocio.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cómo usar esta hoja: completa un renglón por cada proyecto o solicitud nueva (columnas en amarillo). 'Fase de desarrollo' muestra en qué momento del ciclo va cada proyecto (por iniciar, en desarrollo, en pruebas de calidad, en producción en observación, o en producción estable) — junto con 'Estado' y las fechas, responde para cuándo termina y en qué va. 'Fecha real de inicio de desarrollo', 'Fecha real de cierre' y 'Responsable principal' alimentan los indicadores de la hoja 'Resumen' — llénalas a medida que el ítem avanza, no al crearlo. Las 5 filas en azul claro son ejemplos — bórralas o reemplázalas cuando empieces a registrar proyectos reales. No edites la columna 'Prioridad' ni la matriz de la derecha: se calculan solas.</t>
+    <t xml:space="preserve">Cómo usar esta hoja: completa un renglón por cada proyecto o solicitud nueva (columnas en amarillo). 'Fase de desarrollo' muestra en qué momento del ciclo va cada proyecto (por iniciar, en desarrollo, en pruebas de calidad, en producción en observación, o en producción estable) — junto con 'Estado' y las fechas, responde para cuándo termina y en qué va. 'Fecha real de inicio de desarrollo', 'Fecha real de cierre', 'Responsable de desarrollo' y 'Responsable de QA' alimentan los indicadores de la hoja 'Resumen' — llénalas a medida que el ítem avanza, no al crearlo. Usa una sola persona por columna (la principal responsable de cada frente), no una lista, para que la medición de WIP no tenga ambigüedad. Las 5 filas en azul claro son ejemplos — bórralas o reemplázalas cuando empieces a registrar proyectos reales. No edites la columna 'Prioridad' ni la matriz de la derecha: se calculan solas.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen de avance</t>
@@ -518,7 +521,7 @@
     <t xml:space="preserve">Sobre las personas que hoy tienen al menos 1 ítem activo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cómo usar esta tabla: escribe el nombre de cada persona de tu equipo en la columna Persona (las 2 filas en azul son ejemplo, bórralas). El conteo de ítems activos se toma de la columna 'Responsable principal' de 'Seguimiento de proyectos' — usa una sola persona por ítem ahí, no una lista. Esta tabla es una foto de HOY; para medir tendencia real, repite la foto cada semana en el ritual semanal. Si necesitas más de 8 personas, copia el formato de una fila hacia abajo.</t>
+    <t xml:space="preserve">Cómo usar esta tabla: escribe el nombre de cada persona de tu equipo en la columna Persona (las 2 filas en azul son ejemplo, bórralas). El conteo de ítems activos suma la columna 'Responsable de desarrollo' y la columna 'Responsable de QA' de 'Seguimiento de proyectos' — así una persona de QA cuenta igual que una de desarrollo, y alguien que aparece en ambas columnas de un mismo ítem se cuenta una vez por cada rol. Usa una sola persona por columna en cada ítem, no una lista. Esta tabla es una foto de HOY; para medir tendencia real, repite la foto cada semana en el ritual semanal. Si necesitas más de 8 personas, copia el formato de una fila hacia abajo.</t>
   </si>
   <si>
     <t xml:space="preserve">Roles y gobierno (sección 5 del framework KPS)</t>
@@ -598,7 +601,7 @@
     <numFmt numFmtId="167" formatCode="0.0&quot; días&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0\%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -663,6 +666,12 @@
       <i val="true"/>
       <sz val="9.5"/>
       <color rgb="FF52514E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -804,7 +813,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -845,6 +854,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -853,7 +866,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -865,15 +878,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -889,15 +902,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -913,11 +926,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -937,15 +950,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1306,11 +1311,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="23934050"/>
-        <c:axId val="40487919"/>
+        <c:axId val="93475055"/>
+        <c:axId val="30724622"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="23934050"/>
+        <c:axId val="93475055"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1342,7 +1347,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40487919"/>
+        <c:crossAx val="30724622"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1350,7 +1355,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40487919"/>
+        <c:axId val="30724622"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1392,7 +1397,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23934050"/>
+        <c:crossAx val="93475055"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1705,11 +1710,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="10105970"/>
-        <c:axId val="87350264"/>
+        <c:axId val="22551687"/>
+        <c:axId val="31234237"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10105970"/>
+        <c:axId val="22551687"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1741,7 +1746,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87350264"/>
+        <c:crossAx val="31234237"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1749,7 +1754,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87350264"/>
+        <c:axId val="31234237"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1791,7 +1796,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10105970"/>
+        <c:crossAx val="22551687"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1830,9 +1835,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1655640</xdr:colOff>
+      <xdr:colOff>1654920</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>265320</xdr:rowOff>
+      <xdr:rowOff>264600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1841,7 +1846,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="2664360"/>
-        <a:ext cx="5038920" cy="2496960"/>
+        <a:ext cx="5038200" cy="2496240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1860,9 +1865,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>387000</xdr:colOff>
+      <xdr:colOff>386280</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>265320</xdr:rowOff>
+      <xdr:rowOff>264600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1871,7 +1876,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5497920" y="2664360"/>
-        <a:ext cx="5038920" cy="2496960"/>
+        <a:ext cx="5038200" cy="2496240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2561,7 +2566,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:Y20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
@@ -2579,10 +2584,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2605,6 +2610,14 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -2626,6 +2639,41 @@
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
@@ -2679,57 +2727,62 @@
       <c r="Q4" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="R4" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="11"/>
+      <c r="X4" s="10"/>
+      <c r="Y4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="B5" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="C5" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="D5" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="E5" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="12" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E5,$S$6:$S$8,0),MATCH($F5,$T$5:$V$5,0)),"")</f>
+      <c r="F5" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="G5" s="13" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E5,$T$6:$T$8,0),MATCH($F5,$U$5:$W$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11" t="s">
+      <c r="H5" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11" t="s">
+      <c r="K5" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="S5" s="6" t="s">
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12" t="s">
         <v>92</v>
       </c>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="10"/>
       <c r="T5" s="6" t="s">
         <v>93</v>
       </c>
@@ -2737,210 +2790,235 @@
         <v>94</v>
       </c>
       <c r="V5" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="W5" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="X5" s="10"/>
+      <c r="Y5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6" s="13" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E6,$T$6:$T$8,0),MATCH($F6,$U$5:$W$5,0)),"")</f>
+        <v>Alta</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="14" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="U6" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="V6" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="W6" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="X6" s="10"/>
+      <c r="Y6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="G6" s="12" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E6,$S$6:$S$8,0),MATCH($F6,$T$5:$V$5,0)),"")</f>
+      <c r="G7" s="13" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E7,$T$6:$T$8,0),MATCH($F7,$U$5:$W$5,0)),"")</f>
         <v>Alta</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H7" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="S6" s="13" t="s">
+      <c r="U7" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="V7" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="W7" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="X7" s="10"/>
+      <c r="Y7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="T6" s="14" t="s">
+      <c r="E8" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="13" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E8,$T$6:$T$8,0),MATCH($F8,$U$5:$W$5,0)),"")</f>
+        <v>Alta</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="U8" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="V8" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="W8" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="X8" s="10"/>
+      <c r="Y8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="G9" s="13" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E9,$T$6:$T$8,0),MATCH($F9,$U$5:$W$5,0)),"")</f>
+        <v>Baja</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="K9" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="U6" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="V6" s="14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="G7" s="12" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E7,$S$6:$S$8,0),MATCH($F7,$T$5:$V$5,0)),"")</f>
-        <v>Alta</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="S7" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="T7" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="U7" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="V7" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="G8" s="12" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E8,$S$6:$S$8,0),MATCH($F8,$T$5:$V$5,0)),"")</f>
-        <v>Alta</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="S8" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="T8" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="U8" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="V8" s="14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="G9" s="12" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E9,$S$6:$S$8,0),MATCH($F9,$T$5:$V$5,0)),"")</f>
-        <v>Baja</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="10"/>
+      <c r="Y9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8"/>
@@ -2949,8 +3027,8 @@
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
-      <c r="G10" s="15" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E10,$S$6:$S$8,0),MATCH($F10,$T$5:$V$5,0)),"")</f>
+      <c r="G10" s="16" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E10,$T$6:$T$8,0),MATCH($F10,$U$5:$W$5,0)),"")</f>
         <v/>
       </c>
       <c r="H10" s="7"/>
@@ -2963,12 +3041,16 @@
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
       <c r="Q10" s="8"/>
-      <c r="S10" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="T10" s="9"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="9" t="s">
+        <v>126</v>
+      </c>
       <c r="U10" s="9"/>
       <c r="V10" s="9"/>
+      <c r="W10" s="9"/>
+      <c r="X10" s="10"/>
+      <c r="Y10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8"/>
@@ -2977,8 +3059,8 @@
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="15" t="str">
-        <f aca="false">IFERROR(INDEX($T$6:$V$8,MATCH($E11,$S$6:$S$8,0),MATCH($F11,$T$5:$V$5,0)),"")</f>
+      <c r="G11" s="16" t="str">
+        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E11,$T$6:$T$8,0),MATCH($F11,$U$5:$W$5,0)),"")</f>
         <v/>
       </c>
       <c r="H11" s="7"/>
@@ -2991,20 +3073,45 @@
       <c r="O11" s="8"/>
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
-      <c r="S11" s="9"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="10"/>
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
       <c r="V11" s="9"/>
+      <c r="W11" s="9"/>
+      <c r="X11" s="10"/>
+      <c r="Y11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="S12" s="9"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10"/>
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
       <c r="V12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="W12" s="9"/>
+      <c r="X12" s="10"/>
+      <c r="Y12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3022,18 +3129,211 @@
       <c r="O13" s="9"/>
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
-      <c r="S13" s="9"/>
+      <c r="R13" s="9"/>
+      <c r="S13" s="10"/>
       <c r="T13" s="9"/>
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
+      <c r="W13" s="9"/>
+      <c r="X13" s="10"/>
+      <c r="Y13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10"/>
+      <c r="W14" s="10"/>
+      <c r="X14" s="10"/>
+      <c r="Y14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="10"/>
+      <c r="Y15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="10"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="10"/>
+      <c r="W16" s="10"/>
+      <c r="X16" s="10"/>
+      <c r="Y16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="10"/>
+      <c r="U17" s="10"/>
+      <c r="V17" s="10"/>
+      <c r="W17" s="10"/>
+      <c r="X17" s="10"/>
+      <c r="Y17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10"/>
+      <c r="W18" s="10"/>
+      <c r="X18" s="10"/>
+      <c r="Y18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="10"/>
+      <c r="Y19" s="10"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10"/>
+      <c r="W20" s="10"/>
+      <c r="X20" s="10"/>
+      <c r="Y20" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="S4:V4"/>
-    <mergeCell ref="S10:V13"/>
-    <mergeCell ref="A13:Q13"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="T10:W13"/>
+    <mergeCell ref="A13:R13"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D11" type="list">
@@ -3090,7 +3390,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3105,7 +3405,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3119,213 +3419,213 @@
       <c r="K2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="B4" s="10"/>
-      <c r="D4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="10"/>
+      <c r="B4" s="11"/>
+      <c r="D4" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")/COUNTA('Hoja de ruta'!B5:B14)</f>
         <v>0</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="D5" s="17" t="n">
+      <c r="B5" s="17"/>
+      <c r="D5" s="18" t="n">
         <f aca="false">COUNTA('Seguimiento de proyectos'!A5:A11)</f>
         <v>5</v>
       </c>
-      <c r="E5" s="17"/>
+      <c r="E5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="B8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="B8" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="E8" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="G8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="H8" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="J8" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="K8" s="18" t="s">
-        <v>135</v>
+      <c r="K8" s="19" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="B9" s="20" t="n">
+      <c r="A9" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="21" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")</f>
         <v>0</v>
       </c>
-      <c r="D9" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" s="20" t="n">
+      <c r="D9" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="E9" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Muy alta")</f>
         <v>0</v>
       </c>
-      <c r="G9" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="H9" s="22" t="n">
+      <c r="G9" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="H9" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Completado")</f>
         <v>0</v>
       </c>
-      <c r="J9" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="K9" s="22" t="n">
+      <c r="J9" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="K9" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"Por iniciar")</f>
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"En curso")</f>
         <v>1</v>
       </c>
-      <c r="D10" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="E10" s="20" t="n">
+      <c r="D10" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Alta")</f>
         <v>4</v>
       </c>
-      <c r="G10" s="21" t="s">
+      <c r="G10" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"En curso")</f>
         <v>3</v>
       </c>
-      <c r="J10" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="K10" s="22" t="n">
+      <c r="J10" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="K10" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En desarrollo")</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="B11" s="20" t="n">
+      <c r="A11" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="21" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="D11" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="E11" s="20" t="n">
+      <c r="D11" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Media")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="H11" s="22" t="n">
+      <c r="G11" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="H11" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Bloqueado")</f>
         <v>1</v>
       </c>
-      <c r="J11" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="K11" s="22" t="n">
+      <c r="J11" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="K11" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En pruebas de calidad")</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="21" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"No iniciado")</f>
         <v>9</v>
       </c>
-      <c r="D12" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="E12" s="20" t="n">
+      <c r="D12" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Baja")</f>
         <v>1</v>
       </c>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="H12" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"No iniciado")</f>
         <v>1</v>
       </c>
-      <c r="J12" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="K12" s="22" t="n">
+      <c r="J12" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="K12" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (ventana de observación)")</f>
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G13" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="H13" s="22" t="n">
+      <c r="G13" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="H13" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Cancelado")</f>
         <v>0</v>
       </c>
-      <c r="J13" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="K13" s="22" t="n">
+      <c r="J13" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="K13" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (estable)")</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
+      <c r="A16" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -3339,72 +3639,72 @@
       <c r="K17" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="B19" s="24" t="n">
+      <c r="A19" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="B19" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="25" t="s">
-        <v>142</v>
+      <c r="C19" s="26" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
-        <v>143</v>
+      <c r="A21" s="19" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="B22" s="27" t="str">
+      <c r="A22" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="B22" s="28" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$L$5:$L$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")),"")</f>
         <v/>
       </c>
-      <c r="C22" s="25" t="s">
-        <v>145</v>
+      <c r="C22" s="26" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="B23" s="27" t="str">
+      <c r="A23" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B23" s="28" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$O$5:$O$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")),"")</f>
         <v/>
       </c>
-      <c r="C23" s="25" t="s">
-        <v>147</v>
+      <c r="C23" s="26" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="B24" s="28" t="str">
+      <c r="A24" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B24" s="29" t="str">
         <f aca="false">IFERROR(B23/B22*100,"")</f>
         <v/>
       </c>
-      <c r="C24" s="25" t="s">
-        <v>149</v>
+      <c r="C24" s="26" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="B25" s="28" t="str">
+      <c r="A25" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="B25" s="29" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11&lt;='Seguimiento de proyectos'!$M$5:$M$11))/SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;""))*100,"")</f>
         <v/>
       </c>
-      <c r="C25" s="25" t="s">
-        <v>151</v>
+      <c r="C25" s="26" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -3418,159 +3718,159 @@
       <c r="K27" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
+      <c r="A29" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="s">
-        <v>154</v>
-      </c>
-      <c r="B30" s="30" t="s">
+      <c r="A30" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="B30" s="31" t="s">
         <v>156</v>
       </c>
+      <c r="C30" s="31" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="s">
-        <v>157</v>
-      </c>
-      <c r="B31" s="20" t="n">
-        <f aca="false">IF($A31="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A31" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <f aca="false">IF($A31="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C31" s="20" t="str">
+      <c r="C31" s="21" t="str">
         <f aca="false">IF($A31="","",IF(B31&lt;=$B$19,"Sí","No"))</f>
         <v>Sí</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="B32" s="20" t="n">
-        <f aca="false">IF($A32="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A32" s="32" t="s">
+        <v>159</v>
+      </c>
+      <c r="B32" s="21" t="n">
+        <f aca="false">IF($A32="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C32" s="20" t="str">
+      <c r="C32" s="21" t="str">
         <f aca="false">IF($A32="","",IF(B32&lt;=$B$19,"Sí","No"))</f>
         <v>Sí</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="32"/>
-      <c r="B33" s="20" t="n">
-        <f aca="false">IF($A33="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A33,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A33" s="33"/>
+      <c r="B33" s="21" t="n">
+        <f aca="false">IF($A33="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A33,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A33,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C33" s="20" t="str">
+      <c r="C33" s="21" t="str">
         <f aca="false">IF($A33="","",IF(B33&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="32"/>
-      <c r="B34" s="20" t="n">
-        <f aca="false">IF($A34="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A34,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A34" s="33"/>
+      <c r="B34" s="21" t="n">
+        <f aca="false">IF($A34="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A34,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A34,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C34" s="20" t="str">
+      <c r="C34" s="21" t="str">
         <f aca="false">IF($A34="","",IF(B34&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="32"/>
-      <c r="B35" s="20" t="n">
-        <f aca="false">IF($A35="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A35,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A35" s="33"/>
+      <c r="B35" s="21" t="n">
+        <f aca="false">IF($A35="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A35,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A35,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C35" s="20" t="str">
+      <c r="C35" s="21" t="str">
         <f aca="false">IF($A35="","",IF(B35&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="32"/>
-      <c r="B36" s="20" t="n">
-        <f aca="false">IF($A36="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A36,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A36" s="33"/>
+      <c r="B36" s="21" t="n">
+        <f aca="false">IF($A36="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A36,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A36,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C36" s="20" t="str">
+      <c r="C36" s="21" t="str">
         <f aca="false">IF($A36="","",IF(B36&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="32"/>
-      <c r="B37" s="20" t="n">
-        <f aca="false">IF($A37="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A37,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A37" s="33"/>
+      <c r="B37" s="21" t="n">
+        <f aca="false">IF($A37="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A37,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A37,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C37" s="20" t="str">
+      <c r="C37" s="21" t="str">
         <f aca="false">IF($A37="","",IF(B37&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="32"/>
-      <c r="B38" s="20" t="n">
-        <f aca="false">IF($A38="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A38,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
+      <c r="A38" s="33"/>
+      <c r="B38" s="21" t="n">
+        <f aca="false">IF($A38="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A38,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A38,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
         <v>0</v>
       </c>
-      <c r="C38" s="20" t="str">
+      <c r="C38" s="21" t="str">
         <f aca="false">IF($A38="","",IF(B38&lt;=$B$19,"Sí","No"))</f>
         <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="B40" s="33" t="n">
+      <c r="A40" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B40" s="34" t="n">
         <f aca="false">SUM($B$31:$B$38)</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B41" s="28" t="str">
+      <c r="A41" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B41" s="29" t="str">
         <f aca="false">IFERROR((LARGE($B$31:$B$38,1)+LARGE($B$31:$B$38,2))/SUM($B$31:$B$38)*100,"")</f>
         <v/>
       </c>
-      <c r="C41" s="25" t="s">
-        <v>161</v>
+      <c r="C41" s="26" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="B42" s="28" t="str">
+      <c r="A42" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="B42" s="29" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(($B$31:$B$38&gt;0)*($B$31:$B$38&lt;=$B$19))/SUMPRODUCT(($B$31:$B$38&gt;0)*1)*100,"")</f>
         <v/>
       </c>
-      <c r="C42" s="25" t="s">
-        <v>163</v>
+      <c r="C42" s="26" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
@@ -3616,42 +3916,42 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="34" t="s">
-        <v>165</v>
-      </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
+      <c r="A1" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>32</v>
@@ -3659,62 +3959,62 @@
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
       <c r="E5" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -3722,10 +4022,10 @@
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -3733,10 +4033,10 @@
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -3744,33 +4044,33 @@
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
       <c r="E12" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
       <c r="E13" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>

</xml_diff>

<commit_message>
v1.14.0 — plan-implementacion.xlsx: fase PR, retrabajo, combos
Fase de desarrollo suma "En revision de codigo / PR". Nueva columna Retrabajo (Si/No) con indicador % de retrabajo en Resumen. Linea de trabajo, Responsable, Responsable de desarrollo y Responsable de QA pasan a combos desplegables (fuente: Roles y gobierno y la tabla de capacidad de Resumen). Hoja de ruta suma "Cancelado" en Estado. 51 formulas verificadas sin errores.
</commit_message>
<xml_diff>
--- a/docs/plan-implementacion.xlsx
+++ b/docs/plan-implementacion.xlsx
@@ -14,6 +14,10 @@
     <sheet name="Resumen" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Roles y gobierno" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" name="ListaFlujos" vbProcedure="false">'Roles y gobierno'!$B$9:$B$11</definedName>
+    <definedName function="false" hidden="false" name="ListaPersonas" vbProcedure="false">Resumen!$A$31:$A$38</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -24,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="191">
   <si>
     <t xml:space="preserve">Plantilla de implementación por prioridades — cómo usarla</t>
   </si>
@@ -47,43 +51,43 @@
     <t xml:space="preserve">Hoja 'Hoja de ruta'</t>
   </si>
   <si>
-    <t xml:space="preserve">Los 10 pasos generales de instalar el modelo de trabajo. Ya tiene un ejemplo real en el paso 0 (resaltado en azul claro) para mostrar cómo se ve un paso avanzando.</t>
+    <t xml:space="preserve">Los 10 pasos generales de instalar el modelo de trabajo. Ya tiene un ejemplo real en el paso 0 (resaltado en azul claro) para mostrar cómo se ve un paso avanzando. 'Estado' incluye 'Cancelado', igual que en 'Seguimiento de proyectos', para que las dos hojas usen las mismas opciones.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja 'Seguimiento de proyectos'</t>
   </si>
   <si>
-    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado': incluye 'Cancelado' para lo que se descarta sin completarse), en qué momento del ciclo está (columna 'Fase de desarrollo'), y para cuándo se espera. Cuatro columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre', 'Responsable de desarrollo' y 'Responsable de QA' — alimentan los indicadores automáticos de la hoja 'Resumen'. Tiene 5 filas de ejemplo (resaltadas en azul claro) y 2 filas vacías listas para usar.</t>
+    <t xml:space="preserve">El registro vivo de cada proyecto o solicitud: de dónde viene, qué tan urgente es, qué tan grande es, y una prioridad que se calcula sola combinando esas dos cosas — no a criterio de quién pide más fuerte. 'Línea de trabajo asignada', 'Responsable', 'Responsable de desarrollo' y 'Responsable de QA' son combos desplegables (no texto libre), para estandarizar cómo se escribe cada flujo y cada persona. Además responde tres preguntas de negocio para cada proyecto: en qué estado va (columna 'Estado': incluye 'Cancelado' para lo que se descarta sin completarse), en qué momento del ciclo está (columna 'Fase de desarrollo', que distingue 'en desarrollo' de 'en revisión de código / PR' para que un ítem detenido esperando merge no se confunda con uno activo), y para cuándo se espera. Una columna 'Retrabajo' marca cuando algo regresa de pruebas a desarrollo tras un merge. Cinco columnas adicionales — 'Fecha real de inicio de desarrollo', 'Fecha real de cierre', 'Responsable de desarrollo', 'Responsable de QA' y 'Retrabajo' — alimentan los indicadores automáticos de la hoja 'Resumen'.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja 'Resumen'</t>
   </si>
   <si>
-    <t xml:space="preserve">Un panel visual que se actualiza solo a partir de las otras dos hojas — no se edita directamente. Además del avance general, calcula los indicadores de la sección 9 del framework KPS: Lead time, Cycle time, Eficiencia de flujo, % de entrega a tiempo, Índice de concentración y % de cumplimiento de WIP por persona.</t>
+    <t xml:space="preserve">Un panel visual que se actualiza solo a partir de las otras dos hojas — no se edita directamente, salvo la lista de nombres de personas en la tabla de capacidad y el Tope de WIP. Esa misma lista de nombres alimenta los combos de 'Responsable', 'Responsable de desarrollo' y 'Responsable de QA' de 'Seguimiento de proyectos', para que el nombre se escriba siempre igual y el conteo de WIP no falle por variantes. Además del avance general, calcula los indicadores de la sección 9 del framework KPS: Lead time, Cycle time, Eficiencia de flujo, % de entrega a tiempo, % de retrabajo, Índice de concentración y % de cumplimiento de WIP por persona.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja 'Roles y gobierno'</t>
   </si>
   <si>
-    <t xml:space="preserve">El registro de quién tiene cada rol de gobierno del framework (sección 5) y quién es su respaldo nombrado — para que ninguna regla dependa de una sola persona. Trae los 7 roles del framework ya listados, con una fila de 'Líder de Flujo de Valor' por cada flujo de valor (usa los mismos ejemplos de la hoja 'Seguimiento de proyectos'). Completa 'Titular' y 'Respaldo' con los nombres reales de tu equipo.</t>
+    <t xml:space="preserve">El registro de quién tiene cada rol de gobierno del framework (sección 5) y quién es su respaldo nombrado — para que ninguna regla dependa de una sola persona. Trae los 7 roles del framework ya listados, con una fila de 'Líder de Flujo de Valor' por cada flujo de valor. Esos mismos nombres de flujo (filas 9-11, columna 'Alcance') alimentan el combo de 'Línea de trabajo asignada' en 'Seguimiento de proyectos' — agrega una fila aquí para que un flujo nuevo aparezca allá también. Completa 'Titular' y 'Respaldo' con los nombres reales de tu equipo.</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo se calcula la prioridad</t>
   </si>
   <si>
-    <t xml:space="preserve">Se combinan dos preguntas simples: '¿qué tan grave es si esto se atrasa una semana?' (impacto) y '¿qué tan grande es el esfuerzo?' (tamaño). La combinación da la prioridad automáticamente, según la matriz que está al lado de la tabla en la hoja 'Seguimiento de proyectos' (columnas T a W). Impacto alto + esfuerzo pequeño siempre gana — es la forma más simple de evitar que lo urgente-pero-fácil se quede esperando detrás de algo grande y menos importante.</t>
+    <t xml:space="preserve">Se combinan dos preguntas simples: '¿qué tan grave es si esto se atrasa una semana?' (impacto) y '¿qué tan grande es el esfuerzo?' (tamaño). La combinación da la prioridad automáticamente, según la matriz que está al lado de la tabla en la hoja 'Seguimiento de proyectos' (columnas U a X). Impacto alto + esfuerzo pequeño siempre gana — es la forma más simple de evitar que lo urgente-pero-fácil se quede esperando detrás de algo grande y menos importante.</t>
   </si>
   <si>
     <t xml:space="preserve">Indicadores automáticos (sección 9 del framework)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lead time y Cycle time se calculan solos a partir de 'Fecha estimada de inicio', 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' de cada proyecto Completado. El Índice de concentración y el % de cumplimiento de WIP salen de contar, por persona, cuántos ítems tiene 'En curso' sumando la columna 'Responsable de desarrollo' y la columna 'Responsable de QA' — escribe el nombre de cada persona del equipo (desarrollo y QA) en la tabla de la hoja 'Resumen' para que el cálculo funcione.</t>
+    <t xml:space="preserve">Se calculan solos en la hoja 'Resumen' a partir de lo que llenas en 'Seguimiento de proyectos': Lead time, Cycle time, Eficiencia de flujo, % de entrega a tiempo, % de retrabajo, y una tabla de capacidad por persona (desarrollo + QA) con Índice de concentración y % de cumplimiento de WIP.</t>
   </si>
   <si>
     <t xml:space="preserve">Qué editar</t>
   </si>
   <si>
-    <t xml:space="preserve">Las celdas en amarillo son las que se completan para cada paso, proyecto o rol nuevo. Las celdas en azul claro son ejemplos — bórralos o reemplázalos cuando empieces a usar la plantilla con datos reales. No toques las columnas de prioridad, la matriz, ni la hoja 'Resumen' — se calculan solas, excepto la celda amarilla de 'Tope de WIP por persona' y la lista de nombres de personas, que sí son editables.</t>
+    <t xml:space="preserve">Las celdas en amarillo son las que se completan para cada paso, proyecto o rol nuevo. Las celdas en azul claro son ejemplos — bórralos o reemplázalos cuando empieces a usar la plantilla con datos reales. No toques las columnas de prioridad, la matriz, ni la hoja 'Resumen' — se calculan solas, excepto la celda amarilla de 'Tope de WIP por persona' y la lista de nombres de personas, que sí son editables. Los combos de 'Línea de trabajo' y de personas se editan agregando filas en 'Roles y gobierno' (flujos) o en la tabla de capacidad de 'Resumen' (personas) — no en el combo mismo.</t>
   </si>
   <si>
     <t xml:space="preserve">Sin nombrar herramientas</t>
@@ -275,6 +279,9 @@
     <t xml:space="preserve">Responsable de QA (para indicadores de WIP)</t>
   </si>
   <si>
+    <t xml:space="preserve">Retrabajo (regresó de pruebas a desarrollo)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Matriz de prioridad (no editar — solo consulta)</t>
   </si>
   <si>
@@ -407,7 +414,7 @@
     <t xml:space="preserve">Cómo leerla: impacto alto + esfuerzo pequeño siempre gana. Así lo urgente-pero-rápido de resolver no queda esperando detrás de algo grande y menos importante para el negocio.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cómo usar esta hoja: completa un renglón por cada proyecto o solicitud nueva (columnas en amarillo). 'Fase de desarrollo' muestra en qué momento del ciclo va cada proyecto (por iniciar, en desarrollo, en pruebas de calidad, en producción en observación, o en producción estable) — junto con 'Estado' y las fechas, responde para cuándo termina y en qué va. 'Fecha real de inicio de desarrollo', 'Fecha real de cierre', 'Responsable de desarrollo' y 'Responsable de QA' alimentan los indicadores de la hoja 'Resumen' — llénalas a medida que el ítem avanza, no al crearlo. Usa una sola persona por columna (la principal responsable de cada frente), no una lista, para que la medición de WIP no tenga ambigüedad. Las 5 filas en azul claro son ejemplos — bórralas o reemplázalas cuando empieces a registrar proyectos reales. No edites la columna 'Prioridad' ni la matriz de la derecha: se calculan solas.</t>
+    <t xml:space="preserve">Cómo usar esta hoja: completa un renglón por cada proyecto o solicitud nueva (columnas en amarillo). 'Línea de trabajo asignada', 'Responsable', 'Responsable de desarrollo' y 'Responsable de QA' ahora son combos desplegables — no texto libre — para que el mismo flujo o la misma persona se escriba siempre igual (esto es lo que hace que el conteo de WIP en 'Resumen' no se rompa por variantes de escritura del mismo nombre). Para agregar un flujo de valor nuevo, agrégalo en 'Roles y gobierno' (filas de 'Líder de Flujo de Valor'); para agregar una persona nueva, agrégala en la tabla de capacidad de 'Resumen' — el combo se actualiza solo. 'Fase de desarrollo' muestra en qué momento del ciclo va cada proyecto — incluye 'En revisión de código / PR' como paso propio, para que un ítem detenido esperando revisor o merge se vea distinto de uno realmente en desarrollo activo (no lo dejes en 'En desarrollo' por comodidad). Actualiza esta columna el mismo día que el ítem cambia de fase, no al final de la semana — es la misma regla de visibilidad radical del framework (sección 4). 'Retrabajo' se marca 'Sí' cuando un ítem regresa de pruebas a desarrollo después de un merge; alimenta el indicador de rework de la hoja 'Resumen' (sección 9.5 del framework). 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' alimentan los demás indicadores — llénalas a medida que el ítem avanza, no al crearlo. Las 5 filas en azul claro son ejemplos — bórralas o reemplázalas cuando empieces a registrar proyectos reales. No edites la columna 'Prioridad' ni la matriz de la derecha: se calculan solas.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen de avance</t>
@@ -485,7 +492,13 @@
     <t xml:space="preserve">De los ítems con 'Tiene fecha límite real' ya Completados, % entregado en la fecha o antes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nota: los 4 de arriba quedan vacíos hasta que empieces a llenar 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' en 'Seguimiento de proyectos' — al principio solo tienes fechas estimadas.</t>
+    <t xml:space="preserve">% de ítems con retrabajo (regresaron de pruebas a desarrollo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De todos los ítems registrados, cuántos volvieron de pruebas a desarrollo tras un merge (sección 9.5 del framework). No depende de fechas reales, solo de marcar 'Retrabajo' en 'Seguimiento de proyectos'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: Lead time, Cycle time, Eficiencia de flujo y % de entrega a tiempo quedan vacíos hasta que empieces a llenar 'Fecha real de inicio de desarrollo' y 'Fecha real de cierre' en 'Seguimiento de proyectos' — al principio solo tienes fechas estimadas. El % de retrabajo de arriba no depende de fechas: se activa apenas marques 'Sí' en la columna 'Retrabajo'.</t>
   </si>
   <si>
     <t xml:space="preserve">Capacidad y carga por persona — foto de hoy (sección 9.2)</t>
@@ -1311,11 +1324,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="93475055"/>
-        <c:axId val="30724622"/>
+        <c:axId val="54223770"/>
+        <c:axId val="72005471"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="93475055"/>
+        <c:axId val="54223770"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1347,7 +1360,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30724622"/>
+        <c:crossAx val="72005471"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1355,7 +1368,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30724622"/>
+        <c:axId val="72005471"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1397,7 +1410,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93475055"/>
+        <c:crossAx val="54223770"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1710,11 +1723,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="22551687"/>
-        <c:axId val="31234237"/>
+        <c:axId val="82184122"/>
+        <c:axId val="16537103"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="22551687"/>
+        <c:axId val="82184122"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1746,7 +1759,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31234237"/>
+        <c:crossAx val="16537103"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1754,7 +1767,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31234237"/>
+        <c:axId val="16537103"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1796,7 +1809,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22551687"/>
+        <c:crossAx val="82184122"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1835,9 +1848,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1654920</xdr:colOff>
+      <xdr:colOff>1654200</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>264600</xdr:rowOff>
+      <xdr:rowOff>263880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1846,7 +1859,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="2664360"/>
-        <a:ext cx="5038200" cy="2496240"/>
+        <a:ext cx="5037480" cy="2495520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1865,9 +1878,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>386280</xdr:colOff>
+      <xdr:colOff>385560</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>264600</xdr:rowOff>
+      <xdr:rowOff>263880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1876,7 +1889,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5497920" y="2664360"/>
-        <a:ext cx="5038200" cy="2496240"/>
+        <a:ext cx="5037480" cy="2495520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2547,7 +2560,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F14" type="list">
-      <formula1>"No iniciado,En curso,Completado,Bloqueado"</formula1>
+      <formula1>"No iniciado,En curso,Completado,Bloqueado,Cancelado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2566,7 +2579,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
@@ -2584,10 +2597,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="17" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="20" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="1" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2611,13 +2623,14 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
-      <c r="S1" s="10"/>
+      <c r="S1" s="2"/>
       <c r="T1" s="10"/>
       <c r="U1" s="10"/>
       <c r="V1" s="10"/>
       <c r="W1" s="10"/>
       <c r="X1" s="10"/>
       <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -2640,13 +2653,14 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
-      <c r="S2" s="10"/>
+      <c r="S2" s="3"/>
       <c r="T2" s="10"/>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
       <c r="W2" s="10"/>
       <c r="X2" s="10"/>
       <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10"/>
@@ -2674,6 +2688,7 @@
       <c r="W3" s="10"/>
       <c r="X3" s="10"/>
       <c r="Y3" s="10"/>
+      <c r="Z3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
@@ -2730,62 +2745,63 @@
       <c r="R4" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="S4" s="10"/>
-      <c r="T4" s="11" t="s">
+      <c r="S4" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="U4" s="11"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="11" t="s">
+        <v>84</v>
+      </c>
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
-      <c r="X4" s="10"/>
+      <c r="X4" s="11"/>
       <c r="Y4" s="10"/>
+      <c r="Z4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G5" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E5,$T$6:$T$8,0),MATCH($F5,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E5,$U$6:$U$8,0),MATCH($F5,$V$5:$X$5,0)),"")</f>
         <v>Alta</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I5" s="12"/>
       <c r="J5" s="12" t="s">
         <v>36</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L5" s="12"/>
       <c r="M5" s="12"/>
       <c r="N5" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O5" s="12"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
       <c r="R5" s="12"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="6" t="s">
-        <v>93</v>
-      </c>
+      <c r="S5" s="12"/>
+      <c r="T5" s="10"/>
       <c r="U5" s="6" t="s">
         <v>94</v>
       </c>
@@ -2793,43 +2809,46 @@
         <v>95</v>
       </c>
       <c r="W5" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="X5" s="10"/>
+        <v>96</v>
+      </c>
+      <c r="X5" s="6" t="s">
+        <v>90</v>
+      </c>
       <c r="Y5" s="10"/>
+      <c r="Z5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G6" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E6,$T$6:$T$8,0),MATCH($F6,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E6,$U$6:$U$8,0),MATCH($F6,$V$5:$X$5,0)),"")</f>
         <v>Alta</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I6" s="12"/>
       <c r="J6" s="12" t="s">
         <v>41</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
@@ -2838,187 +2857,191 @@
       <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
       <c r="R6" s="12"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="U6" s="15" t="s">
-        <v>103</v>
+      <c r="S6" s="12"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="14" t="s">
+        <v>89</v>
       </c>
       <c r="V6" s="15" t="s">
         <v>104</v>
       </c>
       <c r="W6" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="X6" s="10"/>
+        <v>105</v>
+      </c>
+      <c r="X6" s="15" t="s">
+        <v>105</v>
+      </c>
       <c r="Y6" s="10"/>
+      <c r="Z6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G7" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E7,$T$6:$T$8,0),MATCH($F7,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E7,$U$6:$U$8,0),MATCH($F7,$V$5:$X$5,0)),"")</f>
         <v>Alta</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="12" t="s">
         <v>36</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
       <c r="N7" s="12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O7" s="12"/>
       <c r="P7" s="12"/>
       <c r="Q7" s="12"/>
       <c r="R7" s="12"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="U7" s="15" t="s">
-        <v>104</v>
+      <c r="S7" s="12"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="14" t="s">
+        <v>101</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="W7" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="X7" s="10"/>
+        <v>113</v>
+      </c>
+      <c r="X7" s="15" t="s">
+        <v>113</v>
+      </c>
       <c r="Y7" s="10"/>
+      <c r="Z7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G8" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E8,$T$6:$T$8,0),MATCH($F8,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E8,$U$6:$U$8,0),MATCH($F8,$V$5:$X$5,0)),"")</f>
         <v>Alta</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I8" s="12"/>
       <c r="J8" s="12" t="s">
         <v>36</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
       <c r="N8" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O8" s="12"/>
       <c r="P8" s="12"/>
       <c r="Q8" s="12"/>
       <c r="R8" s="12"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="U8" s="15" t="s">
-        <v>112</v>
+      <c r="S8" s="12"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="14" t="s">
+        <v>119</v>
       </c>
       <c r="V8" s="15" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="W8" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="X8" s="10"/>
+        <v>120</v>
+      </c>
+      <c r="X8" s="15" t="s">
+        <v>120</v>
+      </c>
       <c r="Y8" s="10"/>
+      <c r="Z8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G9" s="13" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E9,$T$6:$T$8,0),MATCH($F9,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E9,$U$6:$U$8,0),MATCH($F9,$V$5:$X$5,0)),"")</f>
         <v>Baja</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I9" s="12"/>
       <c r="J9" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
       <c r="N9" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O9" s="12"/>
       <c r="P9" s="12"/>
       <c r="Q9" s="12"/>
       <c r="R9" s="12"/>
-      <c r="S9" s="10"/>
+      <c r="S9" s="12"/>
       <c r="T9" s="10"/>
       <c r="U9" s="10"/>
       <c r="V9" s="10"/>
       <c r="W9" s="10"/>
       <c r="X9" s="10"/>
       <c r="Y9" s="10"/>
+      <c r="Z9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8"/>
@@ -3028,7 +3051,7 @@
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="16" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E10,$T$6:$T$8,0),MATCH($F10,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E10,$U$6:$U$8,0),MATCH($F10,$V$5:$X$5,0)),"")</f>
         <v/>
       </c>
       <c r="H10" s="7"/>
@@ -3042,15 +3065,16 @@
       <c r="P10" s="8"/>
       <c r="Q10" s="8"/>
       <c r="R10" s="8"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="U10" s="9"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="9" t="s">
+        <v>127</v>
+      </c>
       <c r="V10" s="9"/>
       <c r="W10" s="9"/>
-      <c r="X10" s="10"/>
+      <c r="X10" s="9"/>
       <c r="Y10" s="10"/>
+      <c r="Z10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8"/>
@@ -3060,7 +3084,7 @@
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
       <c r="G11" s="16" t="str">
-        <f aca="false">IFERROR(INDEX($U$6:$W$8,MATCH($E11,$T$6:$T$8,0),MATCH($F11,$U$5:$W$5,0)),"")</f>
+        <f aca="false">IFERROR(INDEX($V$6:$X$8,MATCH($E11,$U$6:$U$8,0),MATCH($F11,$V$5:$X$5,0)),"")</f>
         <v/>
       </c>
       <c r="H11" s="7"/>
@@ -3074,13 +3098,14 @@
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
       <c r="R11" s="8"/>
-      <c r="S11" s="10"/>
-      <c r="T11" s="9"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="10"/>
       <c r="U11" s="9"/>
       <c r="V11" s="9"/>
       <c r="W11" s="9"/>
-      <c r="X11" s="10"/>
+      <c r="X11" s="9"/>
       <c r="Y11" s="10"/>
+      <c r="Z11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10"/>
@@ -3102,16 +3127,17 @@
       <c r="Q12" s="10"/>
       <c r="R12" s="10"/>
       <c r="S12" s="10"/>
-      <c r="T12" s="9"/>
+      <c r="T12" s="10"/>
       <c r="U12" s="9"/>
       <c r="V12" s="9"/>
       <c r="W12" s="9"/>
-      <c r="X12" s="10"/>
+      <c r="X12" s="9"/>
       <c r="Y12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3130,13 +3156,14 @@
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
-      <c r="S13" s="10"/>
-      <c r="T13" s="9"/>
+      <c r="S13" s="9"/>
+      <c r="T13" s="10"/>
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
       <c r="W13" s="9"/>
-      <c r="X13" s="10"/>
+      <c r="X13" s="9"/>
       <c r="Y13" s="10"/>
+      <c r="Z13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10"/>
@@ -3164,6 +3191,7 @@
       <c r="W14" s="10"/>
       <c r="X14" s="10"/>
       <c r="Y14" s="10"/>
+      <c r="Z14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10"/>
@@ -3191,6 +3219,7 @@
       <c r="W15" s="10"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="10"/>
+      <c r="Z15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10"/>
@@ -3218,6 +3247,7 @@
       <c r="W16" s="10"/>
       <c r="X16" s="10"/>
       <c r="Y16" s="10"/>
+      <c r="Z16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10"/>
@@ -3245,6 +3275,7 @@
       <c r="W17" s="10"/>
       <c r="X17" s="10"/>
       <c r="Y17" s="10"/>
+      <c r="Z17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10"/>
@@ -3272,6 +3303,7 @@
       <c r="W18" s="10"/>
       <c r="X18" s="10"/>
       <c r="Y18" s="10"/>
+      <c r="Z18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10"/>
@@ -3299,6 +3331,7 @@
       <c r="W19" s="10"/>
       <c r="X19" s="10"/>
       <c r="Y19" s="10"/>
+      <c r="Z19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10"/>
@@ -3326,16 +3359,17 @@
       <c r="W20" s="10"/>
       <c r="X20" s="10"/>
       <c r="Y20" s="10"/>
+      <c r="Z20" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="T10:W13"/>
-    <mergeCell ref="A13:R13"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="U4:X4"/>
+    <mergeCell ref="U10:X13"/>
+    <mergeCell ref="A13:S13"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="10">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D11" type="list">
       <formula1>"Urgente ahora,Tiene fecha límite real,Puede esperar y priorizarse,Es mantenimiento o mejora interna"</formula1>
       <formula2>0</formula2>
@@ -3353,7 +3387,27 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K11" type="list">
-      <formula1>"Por iniciar,En desarrollo,En pruebas de calidad,En producción (ventana de observación),En producción (estable)"</formula1>
+      <formula1>"Por iniciar,En desarrollo,En revisión de código / PR,En pruebas de calidad,En producción (ventana de observación),En producción (estable)"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="S5:S11" type="list">
+      <formula1>"No,Sí"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H11" type="list">
+      <formula1>ListaFlujos</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I11" type="list">
+      <formula1>ListaPersonas</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q5:Q11" type="list">
+      <formula1>ListaPersonas</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="R5:R11" type="list">
+      <formula1>ListaPersonas</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3390,7 +3444,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3405,7 +3459,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3420,11 +3474,11 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B4" s="11"/>
       <c r="D4" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E4" s="11"/>
     </row>
@@ -3448,54 +3502,54 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>75</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J8" s="19" t="s">
         <v>77</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B9" s="21" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Completado")</f>
         <v>0</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E9" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Muy alta")</f>
         <v>0</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H9" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Completado")</f>
         <v>0</v>
       </c>
       <c r="J9" s="22" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K9" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"Por iniciar")</f>
@@ -3511,7 +3565,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E10" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Alta")</f>
@@ -3525,7 +3579,7 @@
         <v>3</v>
       </c>
       <c r="J10" s="22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K10" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En desarrollo")</f>
@@ -3534,28 +3588,28 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B11" s="21" t="n">
         <f aca="false">COUNTIF('Hoja de ruta'!F5:F14,"Bloqueado")</f>
         <v>0</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Media")</f>
         <v>0</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H11" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Bloqueado")</f>
         <v>1</v>
       </c>
       <c r="J11" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K11" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En pruebas de calidad")</f>
@@ -3571,7 +3625,7 @@
         <v>9</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E12" s="21" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$G$5:$G$11,"Baja")</f>
@@ -3585,7 +3639,7 @@
         <v>1</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K12" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (ventana de observación)")</f>
@@ -3594,14 +3648,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G13" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H13" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$J$5:$J$11,"Cancelado")</f>
         <v>0</v>
       </c>
       <c r="J13" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K13" s="23" t="n">
         <f aca="false">COUNTIF('Seguimiento de proyectos'!$K$5:$K$11,"En producción (estable)")</f>
@@ -3610,7 +3664,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B16" s="24"/>
       <c r="C16" s="24"/>
@@ -3625,7 +3679,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -3640,71 +3694,83 @@
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B19" s="25" t="n">
         <v>2</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B22" s="28" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$L$5:$L$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$L$5:$L$11&lt;&gt;"")),"")</f>
         <v/>
       </c>
       <c r="C22" s="26" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B23" s="28" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11-'Seguimiento de proyectos'!$O$5:$O$11))/SUMPRODUCT(('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$O$5:$O$11&lt;&gt;"")),"")</f>
         <v/>
       </c>
       <c r="C23" s="26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="27" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B24" s="29" t="str">
         <f aca="false">IFERROR(B23/B22*100,"")</f>
         <v/>
       </c>
       <c r="C24" s="26" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B25" s="29" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;"")*('Seguimiento de proyectos'!$P$5:$P$11&lt;='Seguimiento de proyectos'!$M$5:$M$11))/SUMPRODUCT(('Seguimiento de proyectos'!$D$5:$D$11="Tiene fecha límite real")*('Seguimiento de proyectos'!$J$5:$J$11="Completado")*('Seguimiento de proyectos'!$P$5:$P$11&lt;&gt;"")*('Seguimiento de proyectos'!$M$5:$M$11&lt;&gt;""))*100,"")</f>
         <v/>
       </c>
       <c r="C25" s="26" t="s">
-        <v>152</v>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="B26" s="27" t="n">
+        <f aca="false">IFERROR(COUNTIF('Seguimiento de proyectos'!$S$5:$S$11,"Sí")/COUNTA('Seguimiento de proyectos'!$A$5:$A$11)*100,"")</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="26" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -3719,7 +3785,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -3734,18 +3800,18 @@
     </row>
     <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="30" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B30" s="31" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B31" s="21" t="n">
         <f aca="false">IF($A31="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A31,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
@@ -3758,7 +3824,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B32" s="21" t="n">
         <f aca="false">IF($A32="",0,IFERROR(COUNTIFS('Seguimiento de proyectos'!$Q$5:$Q$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso")+COUNTIFS('Seguimiento de proyectos'!$R$5:$R$11,$A32,'Seguimiento de proyectos'!$J$5:$J$11,"En curso"),0))</f>
@@ -3837,7 +3903,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B40" s="34" t="n">
         <f aca="false">SUM($B$31:$B$38)</f>
@@ -3846,31 +3912,31 @@
     </row>
     <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="27" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B41" s="29" t="str">
         <f aca="false">IFERROR((LARGE($B$31:$B$38,1)+LARGE($B$31:$B$38,2))/SUM($B$31:$B$38)*100,"")</f>
         <v/>
       </c>
       <c r="C41" s="26" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="27" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B42" s="29" t="str">
         <f aca="false">IFERROR(SUMPRODUCT(($B$31:$B$38&gt;0)*($B$31:$B$38&lt;=$B$19))/SUMPRODUCT(($B$31:$B$38&gt;0)*1)*100,"")</f>
         <v/>
       </c>
       <c r="C42" s="26" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
@@ -3924,7 +3990,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3933,7 +3999,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3942,16 +4008,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>32</v>
@@ -3959,62 +4025,62 @@
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
       <c r="E5" s="7" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="7" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -4022,10 +4088,10 @@
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -4033,10 +4099,10 @@
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -4044,33 +4110,33 @@
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
       <c r="E12" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
       <c r="E13" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>

</xml_diff>